<commit_message>
fix for single API read
</commit_message>
<xml_diff>
--- a/winner_final/data/spain.xlsx
+++ b/winner_final/data/spain.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dkdk1\PycharmProjects\PythonProjectNew\winner_final\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C31348-F428-4B83-993B-B71DC2850FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B71045-34EC-4B68-BE44-DD09D46C7335}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1995" yWindow="-10860" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2955" yWindow="-14205" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>Team</t>
   </si>
@@ -165,6 +165,9 @@
   </si>
   <si>
     <t>בטיס</t>
+  </si>
+  <si>
+    <t>אלאבס</t>
   </si>
 </sst>
 </file>
@@ -508,7 +511,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.875" customWidth="1"/>
@@ -555,7 +558,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="1" t="s">
@@ -701,6 +704,9 @@
       <c r="C21" t="s">
         <v>21</v>
       </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>